<commit_message>
QMD for new JSON source created
</commit_message>
<xml_diff>
--- a/2Reg_Dictionary_tidy.xlsx
+++ b/2Reg_Dictionary_tidy.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olgau\Documents\Test1\2Reg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FE95A3F-2D78-40F8-99B2-947931CA0E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E6C067-0C94-404D-A9CC-FDA9C27AD255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1420" windowWidth="16640" windowHeight="9380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" refMode="R1C1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="164">
   <si>
     <t>short</t>
   </si>
@@ -506,6 +506,12 @@
   </si>
   <si>
     <t>HA_adverse_effects</t>
+  </si>
+  <si>
+    <t>organization</t>
+  </si>
+  <si>
+    <t>Центр</t>
   </si>
 </sst>
 </file>
@@ -561,8 +567,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:D79" totalsRowShown="0">
-  <autoFilter ref="A1:D79" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:D80" totalsRowShown="0">
+  <autoFilter ref="A1:D80" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="short"/>
     <tableColumn id="4" xr3:uid="{B6680E8C-A5C2-4D72-99F8-F5B2310AAFF4}" name="dataset"/>
@@ -852,7 +858,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.90625" bestFit="1" customWidth="1"/>
@@ -933,13 +939,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
         <v>140</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>163</v>
       </c>
       <c r="D6" t="s">
         <v>4</v>
@@ -947,13 +953,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
         <v>140</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
         <v>4</v>
@@ -961,13 +967,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
         <v>140</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
         <v>4</v>
@@ -975,13 +981,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
         <v>140</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
         <v>4</v>
@@ -989,13 +995,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
         <v>140</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" t="s">
         <v>4</v>
@@ -1003,13 +1009,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>140</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
         <v>4</v>
@@ -1017,13 +1023,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
         <v>140</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
         <v>4</v>
@@ -1031,13 +1037,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
         <v>140</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
         <v>4</v>
@@ -1045,13 +1051,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
         <v>140</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D14" t="s">
         <v>4</v>
@@ -1059,13 +1065,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
         <v>140</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D15" t="s">
         <v>4</v>
@@ -1073,13 +1079,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
         <v>140</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D16" t="s">
         <v>4</v>
@@ -1087,13 +1093,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
         <v>140</v>
       </c>
       <c r="C17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
         <v>4</v>
@@ -1101,27 +1107,27 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
         <v>140</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D18" t="s">
-        <v>35</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B19" t="s">
         <v>140</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
         <v>35</v>
@@ -1129,13 +1135,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
         <v>140</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D20" t="s">
         <v>35</v>
@@ -1143,13 +1149,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B21" t="s">
         <v>140</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D21" t="s">
         <v>35</v>
@@ -1157,13 +1163,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B22" t="s">
         <v>140</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D22" t="s">
         <v>35</v>
@@ -1171,13 +1177,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B23" t="s">
         <v>140</v>
       </c>
       <c r="C23" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D23" t="s">
         <v>35</v>
@@ -1185,13 +1191,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B24" t="s">
         <v>140</v>
       </c>
       <c r="C24" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
         <v>35</v>
@@ -1199,13 +1205,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B25" t="s">
         <v>140</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D25" t="s">
         <v>35</v>
@@ -1213,13 +1219,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B26" t="s">
         <v>140</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D26" t="s">
         <v>35</v>
@@ -1227,13 +1233,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B27" t="s">
         <v>140</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D27" t="s">
         <v>35</v>
@@ -1241,13 +1247,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B28" t="s">
         <v>140</v>
       </c>
       <c r="C28" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D28" t="s">
         <v>35</v>
@@ -1255,13 +1261,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B29" t="s">
         <v>140</v>
       </c>
       <c r="C29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D29" t="s">
         <v>35</v>
@@ -1269,13 +1275,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B30" t="s">
         <v>140</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D30" t="s">
         <v>35</v>
@@ -1283,13 +1289,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B31" t="s">
         <v>140</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D31" t="s">
         <v>35</v>
@@ -1297,13 +1303,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B32" t="s">
         <v>140</v>
       </c>
       <c r="C32" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D32" t="s">
         <v>35</v>
@@ -1311,13 +1317,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B33" t="s">
         <v>140</v>
       </c>
       <c r="C33" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1325,13 +1331,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
         <v>140</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D34" t="s">
         <v>35</v>
@@ -1339,13 +1345,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B35" t="s">
         <v>140</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D35" t="s">
         <v>35</v>
@@ -1353,13 +1359,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B36" t="s">
         <v>140</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D36" t="s">
         <v>35</v>
@@ -1367,13 +1373,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B37" t="s">
         <v>140</v>
       </c>
       <c r="C37" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D37" t="s">
         <v>35</v>
@@ -1381,27 +1387,27 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B38" t="s">
         <v>140</v>
       </c>
       <c r="C38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D38" t="s">
-        <v>4</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B39" t="s">
         <v>140</v>
       </c>
       <c r="C39" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D39" t="s">
         <v>4</v>
@@ -1409,13 +1415,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
         <v>140</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D40" t="s">
         <v>4</v>
@@ -1423,13 +1429,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
         <v>140</v>
       </c>
       <c r="C41" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D41" t="s">
         <v>4</v>
@@ -1437,13 +1443,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B42" t="s">
         <v>140</v>
       </c>
       <c r="C42" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D42" t="s">
         <v>4</v>
@@ -1451,13 +1457,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B43" t="s">
         <v>140</v>
       </c>
       <c r="C43" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D43" t="s">
         <v>4</v>
@@ -1465,13 +1471,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B44" t="s">
         <v>140</v>
       </c>
       <c r="C44" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D44" t="s">
         <v>4</v>
@@ -1479,13 +1485,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B45" t="s">
         <v>140</v>
       </c>
       <c r="C45" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D45" t="s">
         <v>4</v>
@@ -1493,13 +1499,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B46" t="s">
         <v>140</v>
       </c>
       <c r="C46" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D46" t="s">
         <v>4</v>
@@ -1507,13 +1513,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B47" t="s">
         <v>140</v>
       </c>
       <c r="C47" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D47" t="s">
         <v>4</v>
@@ -1521,13 +1527,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B48" t="s">
         <v>140</v>
       </c>
       <c r="C48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D48" t="s">
         <v>4</v>
@@ -1535,13 +1541,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B49" t="s">
         <v>140</v>
       </c>
       <c r="C49" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D49" t="s">
         <v>4</v>
@@ -1549,13 +1555,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B50" t="s">
         <v>140</v>
       </c>
       <c r="C50" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D50" t="s">
         <v>4</v>
@@ -1563,13 +1569,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B51" t="s">
         <v>140</v>
       </c>
       <c r="C51" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D51" t="s">
         <v>4</v>
@@ -1577,13 +1583,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B52" t="s">
         <v>140</v>
       </c>
       <c r="C52" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D52" t="s">
         <v>4</v>
@@ -1591,13 +1597,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B53" t="s">
         <v>140</v>
       </c>
       <c r="C53" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D53" t="s">
         <v>4</v>
@@ -1605,13 +1611,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B54" t="s">
         <v>140</v>
       </c>
       <c r="C54" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D54" t="s">
         <v>4</v>
@@ -1619,13 +1625,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B55" t="s">
         <v>140</v>
       </c>
       <c r="C55" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D55" t="s">
         <v>4</v>
@@ -1633,13 +1639,13 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B56" t="s">
         <v>140</v>
       </c>
       <c r="C56" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D56" t="s">
         <v>4</v>
@@ -1647,13 +1653,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B57" t="s">
         <v>140</v>
       </c>
       <c r="C57" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D57" t="s">
         <v>4</v>
@@ -1661,13 +1667,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B58" t="s">
         <v>140</v>
       </c>
       <c r="C58" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D58" t="s">
         <v>4</v>
@@ -1675,13 +1681,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B59" t="s">
         <v>140</v>
       </c>
       <c r="C59" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D59" t="s">
         <v>4</v>
@@ -1689,13 +1695,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B60" t="s">
         <v>140</v>
       </c>
       <c r="C60" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D60" t="s">
         <v>4</v>
@@ -1703,13 +1709,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B61" t="s">
         <v>140</v>
       </c>
       <c r="C61" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D61" t="s">
         <v>4</v>
@@ -1717,13 +1723,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B62" t="s">
         <v>140</v>
       </c>
       <c r="C62" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D62" t="s">
         <v>4</v>
@@ -1731,13 +1737,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B63" t="s">
         <v>140</v>
       </c>
       <c r="C63" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D63" t="s">
         <v>4</v>
@@ -1745,13 +1751,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B64" t="s">
         <v>140</v>
       </c>
       <c r="C64" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D64" t="s">
         <v>4</v>
@@ -1759,13 +1765,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B65" t="s">
         <v>140</v>
       </c>
       <c r="C65" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D65" t="s">
         <v>4</v>
@@ -1773,13 +1779,13 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B66" t="s">
         <v>140</v>
       </c>
       <c r="C66" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D66" t="s">
         <v>4</v>
@@ -1787,13 +1793,13 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B67" t="s">
         <v>140</v>
       </c>
       <c r="C67" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D67" t="s">
         <v>4</v>
@@ -1801,13 +1807,13 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B68" t="s">
         <v>140</v>
       </c>
       <c r="C68" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D68" t="s">
         <v>4</v>
@@ -1815,13 +1821,13 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C69" t="s">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="D69" t="s">
         <v>4</v>
@@ -1829,13 +1835,13 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="B70" t="s">
         <v>141</v>
       </c>
       <c r="C70" t="s">
-        <v>142</v>
+        <v>3</v>
       </c>
       <c r="D70" t="s">
         <v>4</v>
@@ -1843,13 +1849,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B71" t="s">
         <v>141</v>
       </c>
       <c r="C71" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D71" t="s">
         <v>4</v>
@@ -1857,13 +1863,13 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B72" t="s">
         <v>141</v>
       </c>
       <c r="C72" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D72" t="s">
         <v>4</v>
@@ -1871,13 +1877,13 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B73" t="s">
         <v>141</v>
       </c>
       <c r="C73" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D73" t="s">
         <v>4</v>
@@ -1885,13 +1891,13 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B74" t="s">
         <v>141</v>
       </c>
       <c r="C74" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D74" t="s">
         <v>4</v>
@@ -1899,13 +1905,13 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B75" t="s">
         <v>141</v>
       </c>
       <c r="C75" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D75" t="s">
         <v>4</v>
@@ -1913,13 +1919,13 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B76" t="s">
         <v>141</v>
       </c>
       <c r="C76" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D76" t="s">
         <v>4</v>
@@ -1927,13 +1933,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B77" t="s">
         <v>141</v>
       </c>
       <c r="C77" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D77" t="s">
         <v>4</v>
@@ -1941,13 +1947,13 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B78" t="s">
         <v>141</v>
       </c>
       <c r="C78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D78" t="s">
         <v>4</v>
@@ -1955,15 +1961,29 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B79" t="s">
         <v>141</v>
       </c>
       <c r="C79" t="s">
+        <v>150</v>
+      </c>
+      <c r="D79" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>161</v>
+      </c>
+      <c r="B80" t="s">
+        <v>141</v>
+      </c>
+      <c r="C80" t="s">
         <v>151</v>
       </c>
-      <c r="D79" t="s">
+      <c r="D80" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>